<commit_message>
feat: amazon_asin_database.xlsx 添加 3 条 ASIN 数据及表头冻结 Co-authored-by: monkeycode-ai <monkeycode-ai@chaitin.com>
</commit_message>
<xml_diff>
--- a/resources/userdata/amazon_asin_database.xlsx
+++ b/resources/userdata/amazon_asin_database.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="23040" windowHeight="9527" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASIN 数据库" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,26 +12,181 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ASIN 数据库'!$A$1:$F$1</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="144525" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
+  <fonts count="22">
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
       <b val="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="34">
     <fill>
       <patternFill/>
     </fill>
@@ -40,11 +195,198 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C0C0C0"/>
+        <fgColor rgb="FFC0C0C0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -52,18 +394,309 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="22" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="10"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="49">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="货币[0]" xfId="1" builtinId="7"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="2" builtinId="38"/>
+    <cellStyle name="输入" xfId="3" builtinId="20"/>
+    <cellStyle name="货币" xfId="4" builtinId="4"/>
+    <cellStyle name="千位分隔[0]" xfId="5" builtinId="6"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="6" builtinId="39"/>
+    <cellStyle name="差" xfId="7" builtinId="27"/>
+    <cellStyle name="千位分隔" xfId="8" builtinId="3"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="9" builtinId="40"/>
+    <cellStyle name="超链接" xfId="10" builtinId="8"/>
+    <cellStyle name="百分比" xfId="11" builtinId="5"/>
+    <cellStyle name="已访问的超链接" xfId="12" builtinId="9"/>
+    <cellStyle name="注释" xfId="13" builtinId="10"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="14" builtinId="36"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="警告文本" xfId="16" builtinId="11"/>
+    <cellStyle name="标题" xfId="17" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="18" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="19" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="20" builtinId="17"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="21" builtinId="32"/>
+    <cellStyle name="标题 3" xfId="22" builtinId="18"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="23" builtinId="44"/>
+    <cellStyle name="输出" xfId="24" builtinId="21"/>
+    <cellStyle name="计算" xfId="25" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="26" builtinId="23"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="27" builtinId="50"/>
+    <cellStyle name="强调文字颜色 2" xfId="28" builtinId="33"/>
+    <cellStyle name="链接单元格" xfId="29" builtinId="24"/>
+    <cellStyle name="汇总" xfId="30" builtinId="25"/>
+    <cellStyle name="好" xfId="31" builtinId="26"/>
+    <cellStyle name="适中" xfId="32" builtinId="28"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="33" builtinId="46"/>
+    <cellStyle name="强调文字颜色 1" xfId="34" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="35" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="36" builtinId="31"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="37" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="38" builtinId="35"/>
+    <cellStyle name="强调文字颜色 3" xfId="39" builtinId="37"/>
+    <cellStyle name="强调文字颜色 4" xfId="40" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="41" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="42" builtinId="43"/>
+    <cellStyle name="强调文字颜色 5" xfId="43" builtinId="45"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="45" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -416,7 +1049,6 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -426,8 +1058,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="3"/>
+  <cols>
+    <col width="10.1111111111111" customWidth="1" min="1" max="1"/>
+    <col width="11.8888888888889" customWidth="1" min="2" max="2"/>
+    <col width="43.4444444444444" customWidth="1" min="3" max="3"/>
+    <col width="87.2222222222222" customWidth="1" min="4" max="4"/>
+    <col width="65.8888888888889" customWidth="1" min="5" max="5"/>
+    <col width="32.1111111111111" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -461,8 +1101,108 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MEYD-568</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>B083QH5BK3</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.jp/dp/B083QH5BK3</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>妻の残業NTRわたし、旦那に嘘をついて残業しています…。 めぐり 溜池ゴロー [DVD]</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://m.media-amazon.com/images/I/81RF8kIOYML.SL1500.jpg</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>4549831487865</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>JUFE-118</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>B07YZ92ZJF</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.jp/dp/B07YZ92ZJF</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>射精を支配される究極主観JOI 永井マリア Fitch [DVD]</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://m.media-amazon.com/images/I/91QqZTLtsaL.SL1500.jpg</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>4549831451750</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GVG-907</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>B07T2KYJNB</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.jp/dp/B07T2KYJNB</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>姑の卑猥過ぎる巨乳を狙う娘婿 [DVD]</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://m.media-amazon.com/images/I/91X7F-ilfVL.SL1500.jpg</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>姑の卑猥過ぎる巨乳を狙う娘婿</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" display="https://www.amazon.co.jp/dp/B083QH5BK3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" display="https://m.media-amazon.com/images/I/81RF8kIOYML.SL1500.jpg" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" display="https://www.amazon.co.jp/dp/B07YZ92ZJF" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" display="https://m.media-amazon.com/images/I/91QqZTLtsaL.SL1500.jpg" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" display="https://www.amazon.co.jp/dp/B07T2KYJNB" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" display="https://m.media-amazon.com/images/I/91X7F-ilfVL.SL1500.jpg" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>